<commit_message>
EC_v3: rà soát trùng lặp toàn HĐ phần ngầm, gom hậu quả chậm tiến độ, chậm thanh toán về Điều 18; cập nhật bảng đối chiếu
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013kfHyeUKSX8YviAMfNrZNJ
</commit_message>
<xml_diff>
--- a/3. DỰ THẢO HĐ/16.10.2026 Bảng đối chiếu bản sửa HĐ của Phục Hưng.xlsx
+++ b/3. DỰ THẢO HĐ/16.10.2026 Bảng đối chiếu bản sửa HĐ của Phục Hưng.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phương án đàm phán" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Đối chiếu từng điều" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trùng lặp - mâu thuẫn" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gom điều khoản (EC_v3)" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Đối chiếu từng điều'!$A$4:$Q$76</definedName>
@@ -7822,4 +7823,385 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:D20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="80" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>RÀ SOÁT TRÙNG LẶP TOÀN HỢP ĐỒNG – MỖI NỘI DUNG CHỈ QUY ĐỊNH TẠI MỘT ĐIỀU GỐC (BẢN EC_v3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>Nguyên tắc: hậu quả của chậm trễ, vi phạm (tiến độ, thanh toán, thực hiện thay, chấm dứt) chỉ quy định tại Điều 18; các điều khác chỉ dẫn chiếu. Thể hiện bằng track changes tác giả “VNCN E&amp;C - Rà soát trùng lặp” trong file EC_v3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>Nội dung</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>Điều gốc (giữ lại)</t>
+        </is>
+      </c>
+      <c r="D4" s="16" t="inlineStr">
+        <is>
+          <t>Các chỗ trùng đã xóa / thay bằng dẫn chiếu</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="49.5" customHeight="1">
+      <c r="A5" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="19" t="inlineStr">
+        <is>
+          <t>Hậu quả chậm tiến độ (phạt, bồi thường, biện pháp khắc phục, đình chỉ)</t>
+        </is>
+      </c>
+      <c r="C5" s="18" t="inlineStr">
+        <is>
+          <t>Điều 18.3</t>
+        </is>
+      </c>
+      <c r="D5" s="19" t="inlineStr">
+        <is>
+          <t>7.2e (bồi thường, tăng ca) – xóa; 7.3a, b, c – chuyển vào 18.3, 7.3 chỉ còn dẫn chiếu; 18.3 cũ miễn trừ rộng “không do lỗi CĐT, Bên A, bên thứ ba…” – thay bằng “không được gia hạn theo 7.2 điểm f”.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="35" customHeight="1">
+      <c r="A6" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>Bên A tự thực hiện / thuê đơn vị khác thay Bên B</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Điều 18.4 (chi phí quản lý, khấu trừ theo 3.5)</t>
+        </is>
+      </c>
+      <c r="D6" s="19" t="inlineStr">
+        <is>
+          <t>6.3b, 8.2(i), 12.2.5c, 12.2.8, 12.2.11 (2 đoạn), 12.2.12, 7.3c, 18.4 cũ – thay bằng “xử lý theo Điều 18.4”.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="49.5" customHeight="1">
+      <c r="A7" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="19" t="inlineStr">
+        <is>
+          <t>Chậm tạm ứng, chậm thanh toán của Bên A</t>
+        </is>
+      </c>
+      <c r="C7" s="18" t="inlineStr">
+        <is>
+          <t>Điều 18.7 (mới)</t>
+        </is>
+      </c>
+      <c r="D7" s="19" t="inlineStr">
+        <is>
+          <t>Câu “chậm tạm ứng quá 07 ngày → gia hạn” ở 7.2 ngày bắt đầu; đoạn “CĐT chậm thì lùi” ở 10.3.2e; ngưỡng 45 ngày ở 17.1(iii); ngưỡng 60 ngày ở 17.2c – chuyển về 18.7, các chỗ cũ chỉ dẫn chiếu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="35" customHeight="1">
+      <c r="A8" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="19" t="inlineStr">
+        <is>
+          <t>Gia hạn thời gian hoàn thành và chi phí dừng chờ</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>Điều 7.2 điểm f (ký hiệu cũ i)</t>
+        </is>
+      </c>
+      <c r="D8" s="19" t="inlineStr">
+        <is>
+          <t>4.1.2 (đoạn cuối), 15.1b, 16.5, 17.1(ii), 18.3, 18.7 – chỉ dẫn chiếu; bổ sung căn cứ (iv) chậm tạm ứng, (v) tạm dừng theo 17.1(ii) để không còn chỗ nào cho gia hạn ngoài điểm f.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20.5" customHeight="1">
+      <c r="A9" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="19" t="inlineStr">
+        <is>
+          <t>Khấu trừ, bù trừ</t>
+        </is>
+      </c>
+      <c r="C9" s="18" t="inlineStr">
+        <is>
+          <t>Điều 3.5</t>
+        </is>
+      </c>
+      <c r="D9" s="19" t="inlineStr">
+        <is>
+          <t>10.10 (bù trừ) – gộp vào 3.5 rồi xóa; 11.1 “tạm giữ khoản tiền” – xóa (trùng 10.9).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="35" customHeight="1">
+      <c r="A10" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="19" t="inlineStr">
+        <is>
+          <t>Sửa chữa sai sót, phá dỡ làm lại, chịu tổn thất</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>5.6 (nghĩa vụ) và 18.1 (hậu quả)</t>
+        </is>
+      </c>
+      <c r="D10" s="19" t="inlineStr">
+        <is>
+          <t>4.3 (vế sau), 5.7, 5.8, 5.9 – xóa; 5.10 đánh lại thành 5.7.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="35" customHeight="1">
+      <c r="A11" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="19" t="inlineStr">
+        <is>
+          <t>Điều chỉnh tiến độ</t>
+        </is>
+      </c>
+      <c r="C11" s="18" t="inlineStr">
+        <is>
+          <t>Điều 15.1a</t>
+        </is>
+      </c>
+      <c r="D11" s="19" t="inlineStr">
+        <is>
+          <t>7.2f cũ (lập tiến độ điều chỉnh) và vế “điều chỉnh tiến độ theo yêu cầu” ở 7.2c – xóa, nội dung gộp vào 15.1a.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="35" customHeight="1">
+      <c r="A12" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="19" t="inlineStr">
+        <is>
+          <t>Huy động nhân lực, thiết bị theo tiến độ</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>Điều 7.2 điểm b</t>
+        </is>
+      </c>
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>7.2 điểm d cũ – xóa, gộp “bảo đảm Bên A hoàn thành nghĩa vụ theo HĐ thầu chính” vào điểm b. Ký hiệu g, h, i → d, e, f.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="49.5" customHeight="1">
+      <c r="A13" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="19" t="inlineStr">
+        <is>
+          <t>Hồ sơ và thời hạn quyết toán</t>
+        </is>
+      </c>
+      <c r="C13" s="18" t="inlineStr">
+        <is>
+          <t>Điều 19.1</t>
+        </is>
+      </c>
+      <c r="D13" s="19" t="inlineStr">
+        <is>
+          <t>Danh mục hồ sơ quyết toán ở 10.3.2b – xóa, gộp thành phần còn thiếu vào 19.1(ii); thời hạn xem xét 30 ngày (10.3.2b) và 28 ngày (19.1iii) – thống nhất 30 ngày tại 19.1(iii). 10.3.2b chỉ còn tỷ lệ thanh toán 97%/3%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="35" customHeight="1">
+      <c r="A14" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="19" t="inlineStr">
+        <is>
+          <t>Hồ sơ thanh toán chung</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>Điều 10.3.2a (danh mục), 10.5 (nội dung công văn, phiếu giá)</t>
+        </is>
+      </c>
+      <c r="D14" s="19" t="inlineStr">
+        <is>
+          <t>10.5 a, b, c – rút gọn, bỏ phần trùng hóa đơn; dẫn chiếu 10.3.2, 19.1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20.5" customHeight="1">
+      <c r="A15" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="19" t="inlineStr">
+        <is>
+          <t>Thanh toán phát sinh</t>
+        </is>
+      </c>
+      <c r="C15" s="18" t="inlineStr">
+        <is>
+          <t>Điều 10.3.2 (cùng kỳ thanh toán)</t>
+        </is>
+      </c>
+      <c r="D15" s="19" t="inlineStr">
+        <is>
+          <t>13.2 “14 ngày làm việc” – thay bằng thanh toán cùng kỳ theo 10.3.2 (tránh thời hạn thứ hai).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20.5" customHeight="1">
+      <c r="A16" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="19" t="inlineStr">
+        <is>
+          <t>Thanh toán khi chấm dứt do lỗi Bên A</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>Điều 18.6b</t>
+        </is>
+      </c>
+      <c r="D16" s="19" t="inlineStr">
+        <is>
+          <t>17.2d(viii) – xóa, gộp vào 18.6b (trước đây 2 cách tính khác nhau).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20.5" customHeight="1">
+      <c r="A17" s="17" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="19" t="inlineStr">
+        <is>
+          <t>Hoàn trả tiền bảo hành</t>
+        </is>
+      </c>
+      <c r="C17" s="18" t="inlineStr">
+        <is>
+          <t>Điều 10.3.2c</t>
+        </is>
+      </c>
+      <c r="D17" s="19" t="inlineStr">
+        <is>
+          <t>8.2(iii) – rút gọn thành dẫn chiếu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20.5" customHeight="1">
+      <c r="A18" s="17" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="19" t="inlineStr">
+        <is>
+          <t>Điều chỉnh phạm vi công việc</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>Điều 4.1.1</t>
+        </is>
+      </c>
+      <c r="D18" s="19" t="inlineStr">
+        <is>
+          <t>11.1 – thay bằng dẫn chiếu 4.1.1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20.5" customHeight="1">
+      <c r="A19" s="17" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="19" t="inlineStr">
+        <is>
+          <t>Điều kiện công trường</t>
+        </is>
+      </c>
+      <c r="C19" s="18" t="inlineStr">
+        <is>
+          <t>Điều 9.2</t>
+        </is>
+      </c>
+      <c r="D19" s="19" t="inlineStr">
+        <is>
+          <t>12.2.9 – rút gọn thành dẫn chiếu, chỉ giữ ý không gia hạn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20.5" customHeight="1">
+      <c r="A20" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="19" t="inlineStr">
+        <is>
+          <t>Vật liệu do Bên B cung cấp</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>Điều 14.1</t>
+        </is>
+      </c>
+      <c r="D20" s="19" t="inlineStr">
+        <is>
+          <t>9.3c – xóa.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
 </file>
</xml_diff>